<commit_message>
test(samples): the client's sheets carry rows without a URL
The Groups sheet gains three URL-less rows (Reconstitution by its title, Healing
Peptides, which the replica's hub shares with its store category, and a BPC-157
dosing guide no page answers, planned under its level's page), the Entities sheet
a row that names TB-500 by its entity alone and one that names only Tissue repair,
which plans no page. A replica-shaped site proves each match, and the counts,
trails, types, notes and the row budget the workbook tests pin move with them.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/samples/client-sheets.xlsx
+++ b/samples/client-sheets.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="169" uniqueCount="100">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="218" uniqueCount="114">
   <si>
     <t>Root Entity</t>
   </si>
@@ -145,6 +145,24 @@
     <t>how to store peptides (320); peptide storage</t>
   </si>
   <si>
+    <t>Reconstitution</t>
+  </si>
+  <si>
+    <t>peptide reconstitution (590)</t>
+  </si>
+  <si>
+    <t>Healing Peptides</t>
+  </si>
+  <si>
+    <t>healing peptides (1,600)</t>
+  </si>
+  <si>
+    <t>BPC-157 dosing guide</t>
+  </si>
+  <si>
+    <t>bpc 157 dosage (2,900)</t>
+  </si>
+  <si>
     <t>URL</t>
   </si>
   <si>
@@ -284,6 +302,30 @@
   </si>
   <si>
     <t>Shipping rules differ by province</t>
+  </si>
+  <si>
+    <t>E-015</t>
+  </si>
+  <si>
+    <t>Sold as a 5 mg vial</t>
+  </si>
+  <si>
+    <t>E-041</t>
+  </si>
+  <si>
+    <t>Topic</t>
+  </si>
+  <si>
+    <t>Topical Entity</t>
+  </si>
+  <si>
+    <t>Tissue repair</t>
+  </si>
+  <si>
+    <t>Informational</t>
+  </si>
+  <si>
+    <t>What the healing peptides are researched for</t>
   </si>
   <si>
     <t>Parent Product Entity</t>
@@ -694,7 +736,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G9"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="7" width="28" customWidth="1"/>
@@ -905,6 +947,75 @@
       </c>
       <c r="G9" t="s">
         <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>7</v>
+      </c>
+      <c r="B10" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" t="s">
+        <v>8</v>
+      </c>
+      <c r="D10" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" t="s">
+        <v>43</v>
+      </c>
+      <c r="F10" t="s">
+        <v>8</v>
+      </c>
+      <c r="G10" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" t="s">
+        <v>8</v>
+      </c>
+      <c r="D11" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" t="s">
+        <v>45</v>
+      </c>
+      <c r="F11" t="s">
+        <v>8</v>
+      </c>
+      <c r="G11" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>7</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12" t="s">
+        <v>8</v>
+      </c>
+      <c r="D12" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" t="s">
+        <v>47</v>
+      </c>
+      <c r="F12" t="s">
+        <v>8</v>
+      </c>
+      <c r="G12" t="s">
+        <v>48</v>
       </c>
     </row>
   </sheetData>
@@ -929,7 +1040,7 @@
         <v>2</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="D1" s="1" t="s">
         <v>4</v>
@@ -949,16 +1060,16 @@
         <v>12</v>
       </c>
       <c r="C2" t="s">
-        <v>44</v>
+        <v>50</v>
       </c>
       <c r="D2" t="s">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="E2" t="s">
-        <v>46</v>
+        <v>52</v>
       </c>
       <c r="F2" t="s">
-        <v>47</v>
+        <v>53</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -969,16 +1080,16 @@
         <v>12</v>
       </c>
       <c r="C3" t="s">
-        <v>48</v>
+        <v>54</v>
       </c>
       <c r="D3" t="s">
-        <v>49</v>
+        <v>55</v>
       </c>
       <c r="E3" t="s">
-        <v>50</v>
+        <v>56</v>
       </c>
       <c r="F3" t="s">
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -989,36 +1100,36 @@
         <v>25</v>
       </c>
       <c r="C4" t="s">
-        <v>52</v>
+        <v>58</v>
       </c>
       <c r="D4" t="s">
-        <v>53</v>
+        <v>59</v>
       </c>
       <c r="E4" t="s">
-        <v>54</v>
+        <v>60</v>
       </c>
       <c r="F4" t="s">
-        <v>55</v>
+        <v>61</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>56</v>
+        <v>62</v>
       </c>
       <c r="B5" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="C5" t="s">
-        <v>58</v>
+        <v>64</v>
       </c>
       <c r="D5" t="s">
-        <v>59</v>
+        <v>65</v>
       </c>
       <c r="E5" t="s">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="F5" t="s">
-        <v>61</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1029,7 +1140,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N4"/>
+  <dimension ref="A1:N6"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="14" width="28" customWidth="1"/>
@@ -1037,25 +1148,25 @@
   <sheetData>
     <row r="1" spans="1:14" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>62</v>
+        <v>68</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>63</v>
+        <v>69</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>64</v>
+        <v>70</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>1</v>
@@ -1070,27 +1181,27 @@
         <v>5</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
     </row>
     <row r="2" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="B2" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="C2" t="s">
         <v>1</v>
       </c>
       <c r="D2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="E2" t="s">
         <v>7</v>
@@ -1114,7 +1225,7 @@
         <v>7</v>
       </c>
       <c r="L2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="M2" t="s">
         <v>8</v>
@@ -1125,16 +1236,16 @@
     </row>
     <row r="3" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="B3" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C3" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="D3" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="E3" t="s">
         <v>12</v>
@@ -1158,57 +1269,145 @@
         <v>12</v>
       </c>
       <c r="L3" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="M3" t="s">
         <v>8</v>
       </c>
       <c r="N3" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="B4" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C4" t="s">
+        <v>89</v>
+      </c>
+      <c r="D4" t="s">
+        <v>90</v>
+      </c>
+      <c r="E4" t="s">
+        <v>91</v>
+      </c>
+      <c r="F4" t="s">
+        <v>92</v>
+      </c>
+      <c r="G4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H4" t="s">
+        <v>7</v>
+      </c>
+      <c r="I4" t="s">
+        <v>8</v>
+      </c>
+      <c r="J4" t="s">
+        <v>91</v>
+      </c>
+      <c r="K4" t="s">
+        <v>93</v>
+      </c>
+      <c r="L4" t="s">
+        <v>94</v>
+      </c>
+      <c r="M4" t="s">
+        <v>8</v>
+      </c>
+      <c r="N4" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="5" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>96</v>
+      </c>
+      <c r="B5" t="s">
         <v>83</v>
       </c>
-      <c r="D4" t="s">
+      <c r="C5" t="s">
         <v>84</v>
       </c>
-      <c r="E4" t="s">
+      <c r="D5" t="s">
         <v>85</v>
       </c>
-      <c r="F4" t="s">
+      <c r="E5" t="s">
+        <v>25</v>
+      </c>
+      <c r="F5" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" t="s">
+        <v>8</v>
+      </c>
+      <c r="I5" t="s">
+        <v>8</v>
+      </c>
+      <c r="J5" t="s">
+        <v>8</v>
+      </c>
+      <c r="K5" t="s">
+        <v>8</v>
+      </c>
+      <c r="L5" t="s">
         <v>86</v>
       </c>
-      <c r="G4" t="s">
-        <v>7</v>
-      </c>
-      <c r="H4" t="s">
-        <v>7</v>
-      </c>
-      <c r="I4" t="s">
-        <v>8</v>
-      </c>
-      <c r="J4" t="s">
-        <v>85</v>
-      </c>
-      <c r="K4" t="s">
-        <v>87</v>
-      </c>
-      <c r="L4" t="s">
-        <v>88</v>
-      </c>
-      <c r="M4" t="s">
-        <v>8</v>
-      </c>
-      <c r="N4" t="s">
-        <v>89</v>
+      <c r="M5" t="s">
+        <v>8</v>
+      </c>
+      <c r="N5" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="6" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>98</v>
+      </c>
+      <c r="B6" t="s">
+        <v>83</v>
+      </c>
+      <c r="C6" t="s">
+        <v>99</v>
+      </c>
+      <c r="D6" t="s">
+        <v>100</v>
+      </c>
+      <c r="E6" t="s">
+        <v>101</v>
+      </c>
+      <c r="F6" t="s">
+        <v>8</v>
+      </c>
+      <c r="G6" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6" t="s">
+        <v>8</v>
+      </c>
+      <c r="I6" t="s">
+        <v>8</v>
+      </c>
+      <c r="J6" t="s">
+        <v>8</v>
+      </c>
+      <c r="K6" t="s">
+        <v>8</v>
+      </c>
+      <c r="L6" t="s">
+        <v>102</v>
+      </c>
+      <c r="M6" t="s">
+        <v>8</v>
+      </c>
+      <c r="N6" t="s">
+        <v>103</v>
       </c>
     </row>
   </sheetData>
@@ -1227,19 +1426,19 @@
   <sheetData>
     <row r="1" spans="1:5" s="1" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>90</v>
+        <v>104</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>43</v>
+        <v>49</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>91</v>
+        <v>105</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>92</v>
+        <v>106</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>93</v>
+        <v>107</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -1247,16 +1446,16 @@
         <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>94</v>
+        <v>108</v>
       </c>
       <c r="C2" t="s">
         <v>33</v>
       </c>
       <c r="D2" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="E2" t="s">
-        <v>95</v>
+        <v>109</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -1270,10 +1469,10 @@
         <v>16</v>
       </c>
       <c r="D3" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="E3" t="s">
-        <v>96</v>
+        <v>110</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -1281,16 +1480,16 @@
         <v>25</v>
       </c>
       <c r="B4" t="s">
-        <v>97</v>
+        <v>111</v>
       </c>
       <c r="C4" t="s">
-        <v>98</v>
+        <v>112</v>
       </c>
       <c r="D4" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="E4" t="s">
-        <v>99</v>
+        <v>113</v>
       </c>
     </row>
   </sheetData>

</xml_diff>